<commit_message>
feat: implement dynamic filter chips, UI summary, and collapsible filter panel with restoration logic
</commit_message>
<xml_diff>
--- a/outputs/weekly_purchase_report.xlsx
+++ b/outputs/weekly_purchase_report.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Supplier PO Plan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Immediate Actions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Stockout Alerts" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Substitutions" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="BOM Demand Trace" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Slow Moving Watchlist" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Data Quality Notes" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Blocked By Credit" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier PO Plan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Immediate Actions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stockout Alerts" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Substitutions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM Demand Trace" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slow Moving Watchlist" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality Notes" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocked By Credit" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Executive Summary'!$A$1:$B$9</definedName>
@@ -38,13 +38,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -64,7 +67,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -72,13 +75,19 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">

</xml_diff>